<commit_message>
update manual review TP/FP tagging
</commit_message>
<xml_diff>
--- a/data/september strat simulation/latest(for stakeholder)/strat1254_obs/result_20261007_191632(VN_strat1254_hitlog).xlsx
+++ b/data/september strat simulation/latest(for stakeholder)/strat1254_obs/result_20261007_191632(VN_strat1254_hitlog).xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\september strat simulation\latest(for stakeholder)\strat1254_obs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6319B5C-4A46-43A0-86F4-B970CAE30FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:28001_{FFBD9C68-BA12-4CAC-BF58-5C7E3E7CA7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results export" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
   <si>
     <t>vn_service_disruption_hit_order_rate</t>
   </si>
@@ -46,6 +47,39 @@
   </si>
   <si>
     <t>avg_vn_service_disruption_hit_user_cnt</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>strategy name</t>
+  </si>
+  <si>
+    <t>request</t>
+  </si>
+  <si>
+    <t>interception amount</t>
+  </si>
+  <si>
+    <t>effect amount</t>
+  </si>
+  <si>
+    <t>observe amount</t>
+  </si>
+  <si>
+    <t>pv amount</t>
+  </si>
+  <si>
+    <t>uv amount</t>
+  </si>
+  <si>
+    <t>contribution rate</t>
+  </si>
+  <si>
+    <t>hit rate(%)</t>
+  </si>
+  <si>
+    <t>VN - Service Disruption - Rapid Order Placement - Forbid Order Placing</t>
   </si>
 </sst>
 </file>
@@ -81,8 +115,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.5546875" bestFit="1" customWidth="1"/>
@@ -503,8 +538,342 @@
         <v>15</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <f>A2*100</f>
+        <v>2.5336541115912031E-3</v>
+      </c>
+      <c r="B4">
+        <f>B2*100</f>
+        <v>6.4233941728680972E-4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4185B4-EB36-45FB-B111-F13C30984CB6}">
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46294</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>450140</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>7</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>46295</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>957877</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>35</v>
+      </c>
+      <c r="G3">
+        <v>35</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>46296</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>977830</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>27</v>
+      </c>
+      <c r="G4">
+        <v>27</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46297</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5">
+        <v>1031983</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46298</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>885834</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46299</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7">
+        <v>581413</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>75</v>
+      </c>
+      <c r="G7">
+        <v>75</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46300</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8">
+        <v>956492</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>22</v>
+      </c>
+      <c r="G8">
+        <v>22</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46301</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>936464</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>21</v>
+      </c>
+      <c r="G9">
+        <v>21</v>
+      </c>
+      <c r="H9">
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <f>SUM(C2:C9)</f>
+        <v>6778033</v>
+      </c>
+      <c r="F11">
+        <f>SUM(F2:F9)</f>
+        <v>196</v>
+      </c>
+      <c r="G11">
+        <f>F11/C11*100</f>
+        <v>2.8916943898030594E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>